<commit_message>
Update book import fields and validation
This change updates the book import pipeline to parse the new Excel columns for reading/writing status and to treat empty titles as invalid. It also aligns the frontend URL extraction with the revised template layout, refreshes the BookInsert.xlsx template, and removes the obsolete BookInsertSheet template stub.
</commit_message>
<xml_diff>
--- a/API/Utils/Templates/BookInsert.xlsx
+++ b/API/Utils/Templates/BookInsert.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30502"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30516"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DC446684-0F6C-4278-8AF6-9DB73F94292A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{50D9E06A-A795-40CD-ACE9-96EACA6FBBFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Title</t>
   </si>
@@ -61,12 +61,6 @@
   </si>
   <si>
     <t>WritingStatus</t>
-  </si>
-  <si>
-    <t>Author</t>
-  </si>
-  <si>
-    <t>Author2</t>
   </si>
   <si>
     <t>Url</t>
@@ -82,7 +76,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -94,6 +91,20 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFF1FA8C"/>
+      <name val="Consolas"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -116,14 +127,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -436,10 +453,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="24.5703125" customWidth="1"/>
+    <col min="2" max="2" width="31.140625" customWidth="1"/>
+    <col min="5" max="5" width="21.5703125" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" customWidth="1"/>
+    <col min="8" max="8" width="31" customWidth="1"/>
+    <col min="9" max="9" width="40.42578125" customWidth="1"/>
+    <col min="10" max="10" width="24.5703125" customWidth="1"/>
+    <col min="12" max="12" width="14.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -476,15 +503,81 @@
       <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14">
-      <c r="N2" s="1"/>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="D2" s="2"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="4"/>
+      <c r="J2" s="5"/>
+      <c r="L2" s="1"/>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="D3" s="2"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="4"/>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="D4" s="2"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="4"/>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="D5" s="2"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="4"/>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="D6" s="2"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="4"/>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="D7" s="2"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="4"/>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="D8" s="2"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="4"/>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="D9" s="2"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="4"/>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="D10" s="2"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="4"/>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="D11" s="2"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="4"/>
+    </row>
+    <row r="17" spans="7:7">
+      <c r="G17" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>